<commit_message>
Add top 100 YouTubers data and initial requirements document
- Created a new CSV file containing data for the top 100 YouTubers, including details such as country, channel name, category, followers, engagement rates, and income.
- Added a new Word document for the requirements related to the Customer B chart project.
</commit_message>
<xml_diff>
--- a/project1/Libray Color Options.xlsx
+++ b/project1/Libray Color Options.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary\OneDrive\Desktop\Fanshawe College\Programs_3rd_Sem\6. F_8-10_INFO-3171-01 - User Interfaces_Visualization\Project\project1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FC2EDC-2708-4EEE-B747-AFE9BC2B8F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CB84FC-42CC-4EBB-B169-113819563BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="516" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19420" yWindow="-20800" windowWidth="17890" windowHeight="17180" tabRatio="516" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Options" sheetId="1" r:id="rId1"/>
+    <sheet name="Options" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Option1" sheetId="2" r:id="rId2"/>
     <sheet name="Option2" sheetId="3" r:id="rId3"/>
     <sheet name="Option3" sheetId="4" r:id="rId4"/>
@@ -853,13 +853,7 @@
     <xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -890,6 +884,12 @@
     <xf numFmtId="0" fontId="8" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1234,49 +1234,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="26" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="25.8" x14ac:dyDescent="0.95"/>
   <cols>
-    <col min="1" max="1" width="20.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.6328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1015625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.7890625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.62890625" style="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="19.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="1"/>
+    <col min="6" max="7" width="19.47265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.95">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A2" s="29"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.6">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.95">
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.95">
       <c r="A3" s="16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="52" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="75.5" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1317,7 +1317,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="52" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="49.5" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:10" ht="48.9" x14ac:dyDescent="0.95">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -1357,16 +1357,16 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.95">
       <c r="A8" s="2"/>
       <c r="B8" s="5"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.95">
       <c r="A9" s="16" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="52" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="75.5" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="52" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:10" ht="51.6" x14ac:dyDescent="0.95">
       <c r="A12" s="2" t="s">
         <v>3</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="49.5" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:10" ht="48.9" x14ac:dyDescent="0.95">
       <c r="A13" s="2" t="s">
         <v>4</v>
       </c>
@@ -1471,375 +1471,375 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8622B067-DF6C-49A1-9635-CACC054C438C}">
   <dimension ref="A1:I59"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="30" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" style="30" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="30"/>
+    <col min="1" max="1" width="26.62890625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="13.15625" style="29" customWidth="1"/>
+    <col min="3" max="16384" width="8.734375" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:9" ht="25.8" x14ac:dyDescent="0.95">
+      <c r="A1" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A3" s="30" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A3" s="29" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A5" s="30" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A5" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A6" s="30" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A6" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A8" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A11" s="30" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A11" s="29" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A13" s="30" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A13" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A14" s="30" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A14" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A15" s="30" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A15" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A16" s="30" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A16" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A17" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A20" s="29" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A22" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A23" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="29" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A24" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A25" s="30" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A25" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="29" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A26" s="30" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A26" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="29" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A29" s="30" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A29" s="29" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A31" s="30" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A31" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="30" t="s">
+      <c r="B31" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A32" s="30" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A32" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A33" s="30" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A33" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="29" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A34" s="30" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A34" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="45" t="s">
+      <c r="B34" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A35" s="30" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A35" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="29" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A38" s="30" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A38" s="29" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A40" s="30" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A40" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A42" s="30" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A42" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A44" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="30" t="s">
+      <c r="C44" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A45" s="30" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A45" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C45" s="29" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A46" s="30" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A46" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="33" t="s">
+      <c r="B46" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C46" s="30" t="s">
+      <c r="C46" s="29" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A47" s="30" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A47" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="34" t="s">
+      <c r="B47" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="30" t="s">
+      <c r="C47" s="29" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A48" s="30" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A48" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="47" t="s">
+      <c r="B48" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="30" t="s">
+      <c r="C48" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A49" s="30" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A49" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C49" s="30" t="s">
+      <c r="C49" s="29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A52" s="30" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A52" s="29" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A54" s="30" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A54" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A56" s="30" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A56" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B56" s="30" t="s">
+      <c r="B56" s="29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A57" s="30" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A57" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="49" t="s">
+      <c r="B57" s="47" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A58" s="30" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A58" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="46" t="s">
+      <c r="B58" s="44" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A59" s="30" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A59" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="B59" s="44" t="s">
+      <c r="B59" s="42" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1855,375 +1855,375 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B85A3A1-94A6-4D9C-881D-E43F103C98CC}">
   <dimension ref="A1:I59"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="30" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" style="30" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="30"/>
+    <col min="1" max="1" width="26.62890625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="13.15625" style="29" customWidth="1"/>
+    <col min="3" max="16384" width="8.734375" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:9" ht="25.8" x14ac:dyDescent="0.95">
+      <c r="A1" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A3" s="30" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A3" s="29" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A5" s="30" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A5" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A6" s="30" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A6" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A8" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="55" t="s">
         <v>107</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A11" s="30" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A11" s="29" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A13" s="30" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A13" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A14" s="30" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A14" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="58" t="s">
+      <c r="B14" s="56" t="s">
         <v>108</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A15" s="30" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A15" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="57" t="s">
         <v>109</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A16" s="30" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A16" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="60" t="s">
+      <c r="B16" s="58" t="s">
         <v>110</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A17" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A20" s="29" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A22" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A23" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="29" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A24" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A25" s="30" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A25" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="29" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A26" s="30" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A26" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="29" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A29" s="30" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A29" s="29" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A31" s="30" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A31" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="30" t="s">
+      <c r="B31" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A32" s="30" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A32" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A33" s="30" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A33" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="29" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A34" s="30" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A34" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="45" t="s">
+      <c r="B34" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A35" s="30" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A35" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="29" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A38" s="30" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A38" s="29" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A40" s="30" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A40" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A42" s="30" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A42" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A44" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="30" t="s">
+      <c r="C44" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A45" s="30" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A45" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C45" s="29" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A46" s="30" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A46" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="56" t="s">
+      <c r="B46" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="30" t="s">
+      <c r="C46" s="29" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A47" s="30" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A47" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="57" t="s">
+      <c r="B47" s="55" t="s">
         <v>107</v>
       </c>
-      <c r="C47" s="30" t="s">
+      <c r="C47" s="29" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A48" s="30" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A48" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="47" t="s">
+      <c r="B48" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="30" t="s">
+      <c r="C48" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A49" s="30" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A49" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C49" s="30" t="s">
+      <c r="C49" s="29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A52" s="30" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A52" s="29" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A54" s="30" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A54" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A56" s="30" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A56" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B56" s="30" t="s">
+      <c r="B56" s="29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A57" s="30" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A57" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="49" t="s">
+      <c r="B57" s="47" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A58" s="30" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A58" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="46" t="s">
+      <c r="B58" s="44" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A59" s="30" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A59" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="B59" s="44" t="s">
+      <c r="B59" s="42" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2242,375 +2242,375 @@
     <tabColor rgb="FF7D66C5"/>
   </sheetPr>
   <dimension ref="A1:I59"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="26.6328125" style="30" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" style="30" customWidth="1"/>
-    <col min="3" max="16384" width="8.7265625" style="30"/>
+    <col min="1" max="1" width="26.62890625" style="29" customWidth="1"/>
+    <col min="2" max="2" width="13.15625" style="29" customWidth="1"/>
+    <col min="3" max="16384" width="8.734375" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:9" ht="25.8" x14ac:dyDescent="0.95">
+      <c r="A1" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A3" s="30" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A3" s="29" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A5" s="30" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A5" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A6" s="30" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A6" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A8" s="30" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A8" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A11" s="30" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A11" s="29" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A13" s="30" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A13" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A14" s="30" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A14" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="52" t="s">
+      <c r="B14" s="50" t="s">
         <v>103</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A15" s="30" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A15" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.5">
-      <c r="A16" s="30" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.75">
+      <c r="A16" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="54" t="s">
+      <c r="B16" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A17" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A20" s="29" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A22" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A23" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="29" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A24" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A25" s="30" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A25" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="29" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A26" s="30" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A26" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="29" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A29" s="30" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A29" s="29" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A31" s="30" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A31" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="30" t="s">
+      <c r="B31" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A32" s="30" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A32" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A33" s="30" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A33" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="29" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A34" s="30" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A34" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="45" t="s">
+      <c r="B34" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A35" s="30" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A35" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="29" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A38" s="30" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A38" s="29" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A40" s="30" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A40" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A42" s="30" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A42" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A44" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="30" t="s">
+      <c r="C44" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A45" s="30" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A45" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C45" s="29" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A46" s="30" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A46" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="50" t="s">
+      <c r="B46" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="30" t="s">
+      <c r="C46" s="29" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A47" s="30" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A47" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="51" t="s">
+      <c r="B47" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="C47" s="30" t="s">
+      <c r="C47" s="29" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A48" s="30" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A48" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="47" t="s">
+      <c r="B48" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="30" t="s">
+      <c r="C48" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A49" s="30" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A49" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C49" s="30" t="s">
+      <c r="C49" s="29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A52" s="30" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A52" s="29" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A54" s="30" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A54" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A56" s="30" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A56" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="B56" s="30" t="s">
+      <c r="B56" s="29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A57" s="30" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A57" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="49" t="s">
+      <c r="B57" s="47" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A58" s="30" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A58" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="46" t="s">
+      <c r="B58" s="44" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A59" s="30" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A59" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="B59" s="44" t="s">
+      <c r="B59" s="42" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: starting of the project2,
</commit_message>
<xml_diff>
--- a/project1/Libray Color Options.xlsx
+++ b/project1/Libray Color Options.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39CB84FC-42CC-4EBB-B169-113819563BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA330D9-1CB9-4E5F-8D3E-D6141229DA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19420" yWindow="-20800" windowWidth="17890" windowHeight="17180" tabRatio="516" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25580" yWindow="-19270" windowWidth="12980" windowHeight="17180" tabRatio="516" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Options" sheetId="1" state="hidden" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="114">
   <si>
     <t>Analogous Pastel Palette (Color Suggestions)</t>
   </si>
@@ -419,6 +419,12 @@
   </si>
   <si>
     <t>#F7F4FC</t>
+  </si>
+  <si>
+    <t>Primary Background charts</t>
+  </si>
+  <si>
+    <t>Secondary Background charts</t>
   </si>
 </sst>
 </file>
@@ -2552,24 +2558,24 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A48" s="29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B48" s="45" t="s">
         <v>60</v>
       </c>
       <c r="C48" s="29" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A49" s="29" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B49" s="46" t="s">
         <v>9</v>
       </c>
       <c r="C49" s="29" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.75">

</xml_diff>